<commit_message>
Replaces swp with sb and added clear
</commit_message>
<xml_diff>
--- a/CPU_Instruction_Set.xlsx
+++ b/CPU_Instruction_Set.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Reyansh\BOLT-16_CPU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080887A5-803C-469D-A17D-E9D34E1096DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5D23B8-227E-474B-B6A7-FF711DFCAE3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{25FB4FC9-3870-4051-8B39-19FFBC5F0F37}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -685,7 +685,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="str" cm="1">
-        <f t="array" ref="B2:B9">_xlfn.BASE(_xlfn.SEQUENCE(8,1,0),2,5)</f>
+        <f t="array" ref="B2:B10">_xlfn.BASE(_xlfn.SEQUENCE(9,1,0),2,5)</f>
         <v>00000</v>
       </c>
       <c r="C2" t="s">
@@ -866,6 +866,18 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="str">
+        <v>01000</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>60</v>
+      </c>
       <c r="H10" t="s">
         <v>30</v>
       </c>
@@ -899,18 +911,6 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13">
-        <v>10000</v>
-      </c>
-      <c r="C13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" t="s">
-        <v>60</v>
-      </c>
       <c r="H13" t="s">
         <v>33</v>
       </c>

</xml_diff>